<commit_message>
Describe unlabelled contracts in neutral terms
The supply map now describes other smart contracts only as programs that
hold RBNT, with no example types. Data files, summary and PDF rebuilt.
</commit_message>
<xml_diff>
--- a/public/data/RBNT-Holder-Report-Q3-2026-data.xlsx
+++ b/public/data/RBNT-Holder-Report-Q3-2026-data.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-27 06:50 UTC</t>
+          <t>2026-10-27 08:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1234,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="53" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Programs such as trading pools, vesting and multisig contracts. Not labelled.</t>
+          <t>Programs on the chain that hold RBNT. Not labelled.</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">

</xml_diff>